<commit_message>
feat: deploy standalone 3D Web Experience Portfolio to root index.html
</commit_message>
<xml_diff>
--- a/data/JobTracker.xlsx
+++ b/data/JobTracker.xlsx
@@ -910,29 +910,24 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
           <t>Networking</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>APPLIED</t>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 02:58:16</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Dear Hiring Manager at Telekom Malaysia (TM R&amp;D),
-Saya ingin mengemukakan pe...</t>
-        </is>
-      </c>
+          <t>2026-07-24 02:33:23</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr">
         <is>
           <t>https://tm.com.my/careers/JOB-2026-TM01</t>
@@ -1205,7 +1200,7 @@
         <v>12</v>
       </c>
       <c r="C5" s="13" t="n">
-        <v>66</v>
+        <v>63.7</v>
       </c>
     </row>
     <row r="6">
@@ -1215,10 +1210,10 @@
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C6" s="13" t="n">
-        <v>66</v>
+        <v>63.7</v>
       </c>
     </row>
     <row r="7">
@@ -1267,7 +1262,7 @@
         </is>
       </c>
       <c r="B10" s="12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>0</v>

</xml_diff>